<commit_message>
📊 Report update: 17:04
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1426,6 +1426,158 @@
       <c r="H26" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>45.136.131.32:8445</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>750.2</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>38.34.179.14:8450</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>707.72</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>91.121.63.51:1080</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>397.61</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>65.108.203.36:18080</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>1496.94</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>thespeedx_socks4</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2434,6 +2586,158 @@
       <c r="H26" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>45.136.131.32:8445</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>750.2</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>38.34.179.14:8450</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>707.72</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>91.121.63.51:1080</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>397.61</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>65.108.203.36:18080</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>1496.94</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>thespeedx_socks4</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3074,6 +3378,46 @@
       <c r="H13" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>45.136.131.32:8445</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>750.2</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3170,6 +3514,46 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>неизвестен</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>38.34.179.14:8450</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>707.72</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:00:28</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -3250,55 +3634,55 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>thespeedx_http</t>
+          <t>proxymania</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-26T14:59:47.591824</t>
+          <t>2026-03-26T17:00:28.317203</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G3" t="n">
-        <v>0.007692307692307693</v>
+        <v>0.02272727272727273</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>proxymania</t>
+          <t>thespeedx_http</t>
         </is>
       </c>
       <c r="B4" t="b">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-26T15:28:17.318126</t>
+          <t>2026-03-26T14:59:47.591824</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G4" t="n">
-        <v>14.88372093023256</v>
+        <v>0.007692307692307693</v>
       </c>
     </row>
     <row r="5">
@@ -3311,21 +3695,21 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-26T14:57:54.504793</t>
+          <t>2026-03-26T17:00:28.317872</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G5" t="n">
-        <v>2478.317829457364</v>
+        <v>0.007692307692307693</v>
       </c>
     </row>
     <row r="6">
@@ -3469,7 +3853,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3">
@@ -3479,7 +3863,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -3489,7 +3873,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -3499,7 +3883,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -3509,7 +3893,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -3539,7 +3923,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
     </row>
     <row r="10">
@@ -3550,7 +3934,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T15:28:17</t>
+          <t>2026-03-26T17:00:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 17:17
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1578,6 +1578,202 @@
       <c r="H30" t="inlineStr">
         <is>
           <t>thespeedx_socks4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>38.145.208.209:8444</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>340.45</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>38.34.179.27:8451</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>209.66</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>120.92.212.16:7890</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>966.12</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>38.34.179.162:8451</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>999.65</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>163.227.149.135:8080</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>2607.59</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2738,6 +2934,202 @@
       <c r="H30" t="inlineStr">
         <is>
           <t>thespeedx_socks4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>38.145.208.209:8444</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>340.45</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>38.34.179.27:8451</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>209.66</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>120.92.212.16:7890</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>966.12</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>38.34.179.162:8451</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>999.65</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>163.227.149.135:8080</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>2607.59</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
         </is>
       </c>
     </row>
@@ -2864,7 +3256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3418,6 +3810,46 @@
       <c r="H14" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>38.34.179.27:8451</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>209.66</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3554,6 +3986,86 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>38.145.208.209:8444</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>340.45</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>38.34.179.162:8451</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>999.65</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:05:06</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>thespeedx_socks5</t>
         </is>
       </c>
     </row>
@@ -3688,55 +4200,55 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>thespeedx_socks4</t>
+          <t>thespeedx_socks5</t>
         </is>
       </c>
       <c r="B5" t="b">
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-26T17:00:28.317872</t>
+          <t>2026-03-26T17:05:06.378832</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="G5" t="n">
-        <v>0.007692307692307693</v>
+        <v>0.03731343283582089</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>thespeedx_socks5</t>
+          <t>thespeedx_socks4</t>
         </is>
       </c>
       <c r="B6" t="b">
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-03-26T14:57:54.514770</t>
+          <t>2026-03-26T17:00:28.317872</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G6" t="n">
-        <v>1824.426356589147</v>
+        <v>0.007692307692307693</v>
       </c>
     </row>
     <row r="7">
@@ -3853,7 +4365,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -3863,7 +4375,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -3873,7 +4385,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -3883,7 +4395,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -3893,7 +4405,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -3923,7 +4435,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10">
@@ -3934,7 +4446,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T17:00:28</t>
+          <t>2026-03-26T17:05:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 17:22
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -4268,11 +4268,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-03-26T14:57:54.529134</t>
+          <t>2026-03-26T17:17:20.287448</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G7" t="n">
         <v>1801</v>
@@ -4295,14 +4295,14 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-03-26T14:57:54.718788</t>
+          <t>2026-03-26T17:17:20.702123</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G8" t="n">
-        <v>15.04651162790698</v>
+        <v>15.06153846153846</v>
       </c>
     </row>
     <row r="9">
@@ -4322,14 +4322,14 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-03-26T14:57:54.779874</t>
+          <t>2026-03-26T17:17:20.924234</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G9" t="n">
-        <v>97.79069767441861</v>
+        <v>97.72307692307692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Report update: 18:10
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1774,6 +1774,194 @@
       <c r="H35" t="inlineStr">
         <is>
           <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>106.75.15.167:7890</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>992.76</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>89.208.106.138:10808</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>618.41</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>54.36.117.30:3128</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>673.7</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38.145.208.242:8451</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1962.5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>201.182.85.12:999</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>2105.99</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3130,6 +3318,194 @@
       <c r="H35" t="inlineStr">
         <is>
           <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>106.75.15.167:7890</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>992.76</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>89.208.106.138:10808</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>618.41</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>54.36.117.30:3128</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>673.7</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38.145.208.242:8451</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1962.5</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>201.182.85.12:999</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>2105.99</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3850,6 +4226,46 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>38.145.208.242:8451</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1962.5</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -3864,7 +4280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4066,6 +4482,82 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>thespeedx_socks5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>89.208.106.138:10808</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>618.41</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>54.36.117.30:3128</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>673.7</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-03-26 17:22:48</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -4153,21 +4645,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-26T17:00:28.317203</t>
+          <t>2026-03-26T17:22:48.707950</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02272727272727273</v>
+        <v>0.01492537313432836</v>
       </c>
     </row>
     <row r="4">
@@ -4180,21 +4672,21 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-26T14:59:47.591824</t>
+          <t>2026-03-26T17:22:48.710316</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G4" t="n">
-        <v>0.007692307692307693</v>
+        <v>0.02255639097744361</v>
       </c>
     </row>
     <row r="5">
@@ -4365,7 +4857,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -4375,7 +4867,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -4385,7 +4877,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -4395,7 +4887,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -4405,7 +4897,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -4435,7 +4927,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10">
@@ -4446,7 +4938,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T17:05:06</t>
+          <t>2026-03-26T17:22:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 20:03
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1960,6 +1960,154 @@
         </is>
       </c>
       <c r="H40" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>181.78.194.249:999</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>2975.85</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>194.67.99.223:1080</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>532.0700000000001</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>222.184.48.251:22222</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>1453.28</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>13.36.243.194:9899</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>482.25</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -1976,7 +2124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3504,6 +3652,154 @@
         </is>
       </c>
       <c r="H40" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>181.78.194.249:999</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>2975.85</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>194.67.99.223:1080</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>532.0700000000001</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>222.184.48.251:22222</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>1453.28</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>13.36.243.194:9899</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>482.25</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4280,7 +4576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4556,6 +4852,46 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>194.67.99.223:1080</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>532.0700000000001</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-03-26 19:33:10</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4638,55 +4974,55 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>proxymania</t>
+          <t>thespeedx_http</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-26T17:22:48.707950</t>
+          <t>2026-03-26T19:33:10.828732</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01492537313432836</v>
+        <v>0.05109489051094891</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>thespeedx_http</t>
+          <t>proxymania</t>
         </is>
       </c>
       <c r="B4" t="b">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-26T17:22:48.710316</t>
+          <t>2026-03-26T17:22:48.707950</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02255639097744361</v>
+        <v>0.01492537313432836</v>
       </c>
     </row>
     <row r="5">
@@ -4857,7 +5193,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -4867,7 +5203,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -4877,7 +5213,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -4887,7 +5223,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -4897,7 +5233,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -4927,7 +5263,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>253</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10">
@@ -4938,7 +5274,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T17:22:48</t>
+          <t>2026-03-26T19:33:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 20:49
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2108,6 +2108,226 @@
         </is>
       </c>
       <c r="H44" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>38.194.246.34:999</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>2179.36</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>43.99.54.236:5555</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1074.84</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>45.136.130.193:8444</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>1189.26</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1.1.213.177:8080</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>1717.97</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>103.30.29.115:20326</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>1989.71</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>149.40.26.240:8080</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="n">
+        <v>1114.89</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -2124,7 +2344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3800,6 +4020,226 @@
         </is>
       </c>
       <c r="H44" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>38.194.246.34:999</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>2179.36</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>43.99.54.236:5555</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1074.84</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>45.136.130.193:8444</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>1189.26</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>1.1.213.177:8080</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>1717.97</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>103.30.29.115:20326</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>1989.71</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>149.40.26.240:8080</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="n">
+        <v>1114.89</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3928,7 +4368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4562,6 +5002,46 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>43.99.54.236:5555</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1074.84</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:03:49</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -4981,21 +5461,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-26T19:33:10.828732</t>
+          <t>2026-03-26T20:03:49.309042</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G3" t="n">
-        <v>0.05109489051094891</v>
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="4">
@@ -5008,21 +5488,21 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-26T17:22:48.707950</t>
+          <t>2026-03-26T20:03:49.305928</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01492537313432836</v>
+        <v>0.0364963503649635</v>
       </c>
     </row>
     <row r="5">
@@ -5193,7 +5673,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3">
@@ -5203,7 +5683,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -5223,7 +5703,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -5263,7 +5743,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="10">
@@ -5274,7 +5754,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T19:33:10</t>
+          <t>2026-03-26T20:03:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 21:19
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2328,6 +2328,162 @@
         </is>
       </c>
       <c r="H50" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>38.34.179.105:8449</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1028.65</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>38.145.208.240:8446</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>356.11</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>103.156.16.160:8080</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>1664.11</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>121.230.8.220:1080</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1168.11</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -2344,7 +2500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4240,6 +4396,162 @@
         </is>
       </c>
       <c r="H50" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>38.34.179.105:8449</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1028.65</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>38.145.208.240:8446</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>356.11</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>103.156.16.160:8080</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="n">
+        <v>1664.11</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>121.230.8.220:1080</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1168.11</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4368,7 +4680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5040,6 +5352,86 @@
         </is>
       </c>
       <c r="H17" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>38.34.179.105:8449</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1028.65</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>38.145.208.240:8446</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>356.11</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-03-26 20:49:23</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -5431,52 +5823,52 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>неизвестен</t>
+          <t>thespeedx_http</t>
         </is>
       </c>
       <c r="B2" t="b">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T15:28:17.311981</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+          <t>2026-03-26T20:49:23.265533</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>142</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.08450704225352113</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>thespeedx_http</t>
+          <t>неизвестен</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-26T20:03:49.309042</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>140</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.07142857142857142</v>
-      </c>
+          <t>2026-03-26T15:28:17.311981</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5488,21 +5880,21 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-26T20:03:49.305928</t>
+          <t>2026-03-26T20:49:23.264575</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0364963503649635</v>
+        <v>0.05714285714285714</v>
       </c>
     </row>
     <row r="5">
@@ -5673,7 +6065,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3">
@@ -5683,7 +6075,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -5703,7 +6095,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -5743,7 +6135,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>263</v>
+        <v>267</v>
       </c>
     </row>
     <row r="10">
@@ -5754,7 +6146,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T20:03:49</t>
+          <t>2026-03-26T20:49:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 21:50
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2484,6 +2484,154 @@
         </is>
       </c>
       <c r="H54" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>103.144.209.104:8715</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>2039.46</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>65.108.203.35:28080</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="n">
+        <v>941.98</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>38.34.179.40:8446</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>868.99</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>178.156.224.42:3128</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>1791.97</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -2500,7 +2648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4552,6 +4700,154 @@
         </is>
       </c>
       <c r="H54" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>103.144.209.104:8715</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="n">
+        <v>2039.46</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>65.108.203.35:28080</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="n">
+        <v>941.98</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>38.34.179.40:8446</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>868.99</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>178.156.224.42:3128</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="n">
+        <v>1791.97</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4680,7 +4976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5434,6 +5730,46 @@
       <c r="H19" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>38.34.179.40:8446</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>868.99</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:20:07</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -5830,21 +6166,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T20:49:23.265533</t>
+          <t>2026-03-26T21:20:07.529775</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G2" t="n">
-        <v>0.08450704225352113</v>
+        <v>0.1095890410958904</v>
       </c>
     </row>
     <row r="3">
@@ -6065,7 +6401,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -6075,7 +6411,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -6135,7 +6471,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>267</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10">
@@ -6146,7 +6482,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T20:49:23</t>
+          <t>2026-03-26T21:20:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 22:18
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2632,6 +2632,158 @@
         </is>
       </c>
       <c r="H58" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>38.34.183.234:8450</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1546.16</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>119.18.145.52:20326</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>2234.12</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>103.40.226.126:26100</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>2866.2</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>45.136.130.171:8445</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1172.53</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -2648,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4848,6 +5000,158 @@
         </is>
       </c>
       <c r="H58" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>38.34.183.234:8450</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1546.16</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>119.18.145.52:20326</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="n">
+        <v>2234.12</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>103.40.226.126:26100</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="n">
+        <v>2866.2</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>45.136.130.171:8445</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1172.53</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4976,7 +5280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5768,6 +6072,46 @@
         </is>
       </c>
       <c r="H20" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>38.34.183.234:8450</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1546.16</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5784,7 +6128,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6100,6 +6444,46 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>45.136.130.171:8445</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1172.53</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-03-26 21:51:01</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6166,21 +6550,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T21:20:07.529775</t>
+          <t>2026-03-26T21:51:01.217002</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1095890410958904</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -6401,7 +6785,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3">
@@ -6411,7 +6795,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -6421,7 +6805,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -6431,7 +6815,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -6441,7 +6825,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -6471,7 +6855,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>271</v>
+        <v>275</v>
       </c>
     </row>
     <row r="10">
@@ -6482,7 +6866,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T21:20:07</t>
+          <t>2026-03-26T21:51:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 22:52
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2784,6 +2784,198 @@
         </is>
       </c>
       <c r="H62" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>187.49.176.141:8080</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>944.76</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>210.201.86.72:8080</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>858.39</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>101.6.65.26:10808</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1371.17</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>47.77.193.180:1080</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>180.42</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>103.84.95.54:7890</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1973.32</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -2800,7 +2992,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5152,6 +5344,198 @@
         </is>
       </c>
       <c r="H62" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>187.49.176.141:8080</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="n">
+        <v>944.76</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>210.201.86.72:8080</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="n">
+        <v>858.39</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>101.6.65.26:10808</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1371.17</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>47.77.193.180:1080</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>180.42</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>103.84.95.54:7890</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1973.32</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5280,7 +5664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6112,6 +6496,46 @@
         </is>
       </c>
       <c r="H21" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>103.84.95.54:7890</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1973.32</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6128,7 +6552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6484,6 +6908,46 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>47.77.193.180:1080</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>180.42</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:18:34</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6550,21 +7014,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T21:51:01.217002</t>
+          <t>2026-03-26T22:18:34.365517</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1333333333333333</v>
+        <v>0.1612903225806452</v>
       </c>
     </row>
     <row r="3">
@@ -6785,7 +7249,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
@@ -6795,7 +7259,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
@@ -6805,7 +7269,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -6815,7 +7279,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -6825,7 +7289,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -6855,7 +7319,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10">
@@ -6866,7 +7330,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T21:51:01</t>
+          <t>2026-03-26T22:18:34</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 23:28
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2976,6 +2976,122 @@
         </is>
       </c>
       <c r="H67" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>38.145.220.102:8453</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>2523.64</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:05</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:05</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>119.18.144.3:30226</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>1524.19</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>5.104.87.17:8051</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1109.17</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -2992,7 +3108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5536,6 +5652,122 @@
         </is>
       </c>
       <c r="H67" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>38.145.220.102:8453</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>2523.64</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:05</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:05</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>119.18.144.3:30226</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="n">
+        <v>1524.19</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>5.104.87.17:8051</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1109.17</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5664,7 +5896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6536,6 +6768,86 @@
         </is>
       </c>
       <c r="H22" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>38.145.220.102:8453</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2523.64</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:05</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:05</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>5.104.87.17:8051</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1109.17</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-03-26 22:53:06</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7014,21 +7326,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D2" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T22:18:34.365517</t>
+          <t>2026-03-26T22:53:06.002454</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1612903225806452</v>
+        <v>0.1772151898734177</v>
       </c>
     </row>
     <row r="3">
@@ -7249,7 +7561,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
@@ -7259,7 +7571,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4">
@@ -7279,7 +7591,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -7319,7 +7631,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="10">
@@ -7330,7 +7642,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T22:18:34</t>
+          <t>2026-03-26T22:53:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 23:59
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3092,6 +3092,162 @@
         </is>
       </c>
       <c r="H70" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>163.5.128.37:14270</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>678.8200000000001</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>150.107.140.238:3128</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1976.51</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>38.145.208.244:8448</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>198.44</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>167.103.144.127:8800</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>724.85</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3108,7 +3264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5768,6 +5924,162 @@
         </is>
       </c>
       <c r="H70" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>163.5.128.37:14270</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>678.8200000000001</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>150.107.140.238:3128</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1976.51</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>38.145.208.244:8448</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>198.44</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>167.103.144.127:8800</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>724.85</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5896,7 +6208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6848,6 +7160,126 @@
         </is>
       </c>
       <c r="H24" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>150.107.140.238:3128</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1976.51</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>38.145.208.244:8448</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>198.44</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>167.103.144.127:8800</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>AU</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>724.85</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:28:37</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7326,21 +7758,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="D2" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T22:53:06.002454</t>
+          <t>2026-03-26T23:28:37.559337</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1772151898734177</v>
+        <v>0.1975308641975309</v>
       </c>
     </row>
     <row r="3">
@@ -7561,7 +7993,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3">
@@ -7571,7 +8003,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -7591,7 +8023,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -7631,7 +8063,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>283</v>
+        <v>287</v>
       </c>
     </row>
     <row r="10">
@@ -7642,7 +8074,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T22:53:06</t>
+          <t>2026-03-26T23:28:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 03:25
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3248,6 +3248,158 @@
         </is>
       </c>
       <c r="H74" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>203.205.49.2:10014</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2999.7</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>157.20.253.43:8989</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>1909.51</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>86.53.183.16:1080</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>713.54</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>137.220.150.170:6005</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>2806.75</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3264,7 +3416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6080,6 +6232,158 @@
         </is>
       </c>
       <c r="H74" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>203.205.49.2:10014</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="n">
+        <v>2999.7</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>157.20.253.43:8989</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="n">
+        <v>1909.51</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>86.53.183.16:1080</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>713.54</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>137.220.150.170:6005</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>2806.75</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7296,7 +7600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7692,6 +7996,46 @@
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>86.53.183.16:1080</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>713.54</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-03-26 23:59:58</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7758,21 +8102,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D2" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T23:28:37.559337</t>
+          <t>2026-03-26T23:59:58.552534</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1975308641975309</v>
+        <v>0.2168674698795181</v>
       </c>
     </row>
     <row r="3">
@@ -7993,7 +8337,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -8003,7 +8347,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4">
@@ -8013,7 +8357,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -8023,7 +8367,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -8033,7 +8377,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -8063,7 +8407,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>287</v>
+        <v>291</v>
       </c>
     </row>
     <row r="10">
@@ -8074,7 +8418,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T23:28:37</t>
+          <t>2026-03-26T23:59:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 05:23
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3400,6 +3400,86 @@
         </is>
       </c>
       <c r="H78" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>16.78.119.130:443</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1063.16</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>15.204.151.149:3128</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>367.86</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3416,7 +3496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6384,6 +6464,86 @@
         </is>
       </c>
       <c r="H78" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>16.78.119.130:443</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1063.16</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>15.204.151.149:3128</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>367.86</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6512,7 +6672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7584,6 +7744,46 @@
         </is>
       </c>
       <c r="H27" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>15.204.151.149:3128</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>367.86</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-03-27 03:25:45</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -8102,21 +8302,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-26T23:59:58.552534</t>
+          <t>2026-03-27T03:25:45.664910</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2168674698795181</v>
+        <v>0.2261904761904762</v>
       </c>
     </row>
     <row r="3">
@@ -8337,7 +8537,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3">
@@ -8347,7 +8547,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4">
@@ -8407,7 +8607,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="10">
@@ -8418,7 +8618,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-26T23:59:58</t>
+          <t>2026-03-27T03:25:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 06:44
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3480,6 +3480,198 @@
         </is>
       </c>
       <c r="H80" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>195.123.213.129:1080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>2800.34</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>120.92.212.16:8890</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>953.05</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>45.140.147.155:1081</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>525.4</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>57.128.188.167:8188</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>1923.01</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>161.49.90.70:1337</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>2327.23</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3496,7 +3688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H80"/>
+  <dimension ref="A1:H85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6544,6 +6736,198 @@
         </is>
       </c>
       <c r="H80" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>195.123.213.129:1080</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>2800.34</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>120.92.212.16:8890</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>953.05</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>45.140.147.155:1081</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>525.4</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>57.128.188.167:8188</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="n">
+        <v>1923.01</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>161.49.90.70:1337</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="n">
+        <v>2327.23</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6672,7 +7056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7786,6 +8170,46 @@
       <c r="H28" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>195.123.213.129:1080</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>LV</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>2800.34</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-03-27 05:23:21</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -8302,72 +8726,72 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D2" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T03:25:45.664910</t>
+          <t>2026-03-27T05:23:21.647781</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2261904761904762</v>
+        <v>0.2352941176470588</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>неизвестен</t>
+          <t>proxymania</t>
         </is>
       </c>
       <c r="B3" t="b">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-26T15:28:17.311981</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+          <t>2026-03-27T05:23:21.645161</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>143</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.07692307692307693</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>proxymania</t>
+          <t>неизвестен</t>
         </is>
       </c>
       <c r="B4" t="b">
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-26T20:49:23.264575</t>
-        </is>
-      </c>
-      <c r="F4" t="n">
-        <v>140</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.05714285714285714</v>
-      </c>
+          <t>2026-03-26T15:28:17.311981</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8537,7 +8961,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -8547,7 +8971,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
@@ -8567,7 +8991,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -8607,7 +9031,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="10">
@@ -8618,7 +9042,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T03:25:45</t>
+          <t>2026-03-27T05:23:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 07:48
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3672,6 +3672,82 @@
         </is>
       </c>
       <c r="H85" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8126</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>🇷🇺 Россия</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>2800.94</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>59.46.216.131:30001</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="n">
+        <v>1972.41</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3688,7 +3764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6928,6 +7004,82 @@
         </is>
       </c>
       <c r="H85" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8126</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>🇷🇺 Россия</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>2800.94</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>59.46.216.131:30001</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="n">
+        <v>1972.41</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7000,7 +7152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7042,6 +7194,46 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8126</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>🇷🇺 Россия</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2800.94</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-03-27 06:45:05</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -8726,21 +8918,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T05:23:21.647781</t>
+          <t>2026-03-27T06:45:05.104088</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2352941176470588</v>
+        <v>0.239766081871345</v>
       </c>
     </row>
     <row r="3">
@@ -8753,21 +8945,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T05:23:21.645161</t>
+          <t>2026-03-27T06:45:05.102538</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G3" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.08333333333333333</v>
       </c>
     </row>
     <row r="4">
@@ -8961,7 +9153,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3">
@@ -8971,7 +9163,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -9031,7 +9223,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10">
@@ -9042,7 +9234,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T05:23:21</t>
+          <t>2026-03-27T06:45:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 08:35
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3748,6 +3748,162 @@
         </is>
       </c>
       <c r="H87" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>38.34.179.161:8448</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>478.19</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>45.149.92.147:5001</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1050.12</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>114.130.153.46:58080</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="n">
+        <v>1739.08</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>160.250.134.143:3128</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1150.45</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3764,7 +3920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7080,6 +7236,162 @@
         </is>
       </c>
       <c r="H87" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>38.34.179.161:8448</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>478.19</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>45.149.92.147:5001</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1050.12</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>114.130.153.46:58080</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="n">
+        <v>1739.08</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>160.250.134.143:3128</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1150.45</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7248,7 +7560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8402,6 +8714,46 @@
       <c r="H29" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>160.250.134.143:3128</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>VN</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1150.45</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -8416,7 +8768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8854,6 +9206,46 @@
       <c r="H11" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>38.34.179.161:8448</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>478.19</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-03-27 07:48:24</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -8918,21 +9310,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D2" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T06:45:05.104088</t>
+          <t>2026-03-27T07:48:24.140844</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="G2" t="n">
-        <v>0.239766081871345</v>
+        <v>0.2528735632183908</v>
       </c>
     </row>
     <row r="3">
@@ -8945,21 +9337,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T06:45:05.102538</t>
+          <t>2026-03-27T07:48:24.135166</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G3" t="n">
-        <v>0.08333333333333333</v>
+        <v>0.0958904109589041</v>
       </c>
     </row>
     <row r="4">
@@ -9153,7 +9545,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3">
@@ -9163,7 +9555,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
@@ -9173,7 +9565,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5">
@@ -9183,7 +9575,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -9193,7 +9585,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -9223,7 +9615,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="10">
@@ -9234,7 +9626,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T06:45:05</t>
+          <t>2026-03-27T07:48:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 09:37
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3904,6 +3904,82 @@
         </is>
       </c>
       <c r="H91" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8124</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>1131.85</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>137.220.150.152:6005</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>2583.1</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3920,7 +3996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7392,6 +7468,82 @@
         </is>
       </c>
       <c r="H91" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8124</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="n">
+        <v>1131.85</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>137.220.150.152:6005</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>2583.1</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2026-03-27 08:36:11</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9310,21 +9462,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D2" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T07:48:24.140844</t>
+          <t>2026-03-27T08:36:11.783012</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2528735632183908</v>
+        <v>0.2571428571428571</v>
       </c>
     </row>
     <row r="3">
@@ -9337,21 +9489,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T07:48:24.135166</t>
+          <t>2026-03-27T08:36:11.781100</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0958904109589041</v>
+        <v>0.1020408163265306</v>
       </c>
     </row>
     <row r="4">
@@ -9545,7 +9697,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -9555,7 +9707,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4">
@@ -9615,7 +9767,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="10">
@@ -9626,7 +9778,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T07:48:24</t>
+          <t>2026-03-27T08:36:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 10:31
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3980,6 +3980,42 @@
         </is>
       </c>
       <c r="H93" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>163.5.128.129:14270</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="n">
+        <v>2272.15</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-03-27 09:37:29</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-03-27 09:37:29</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -3996,7 +4032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7544,6 +7580,42 @@
         </is>
       </c>
       <c r="H93" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>163.5.128.129:14270</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="n">
+        <v>2272.15</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-03-27 09:37:29</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-03-27 09:37:29</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9462,21 +9534,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D2" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T08:36:11.783012</t>
+          <t>2026-03-27T09:37:29.585114</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2571428571428571</v>
+        <v>0.2613636363636364</v>
       </c>
     </row>
     <row r="3">
@@ -9697,7 +9769,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3">
@@ -9707,7 +9779,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4">
@@ -9767,7 +9839,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10">
@@ -9778,7 +9850,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T08:36:11</t>
+          <t>2026-03-27T09:37:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 11:26
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4016,6 +4016,42 @@
         </is>
       </c>
       <c r="H94" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>120.92.211.211:7890</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>2444.98</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-03-27 10:31:30</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-03-27 10:31:30</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4032,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7616,6 +7652,42 @@
         </is>
       </c>
       <c r="H94" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>120.92.211.211:7890</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="n">
+        <v>2444.98</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-03-27 10:31:30</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-03-27 10:31:30</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9534,21 +9606,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D2" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T09:37:29.585114</t>
+          <t>2026-03-27T10:31:30.075994</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2613636363636364</v>
+        <v>0.2655367231638418</v>
       </c>
     </row>
     <row r="3">
@@ -9769,7 +9841,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -9779,7 +9851,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4">
@@ -9839,7 +9911,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="10">
@@ -9850,7 +9922,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T09:37:29</t>
+          <t>2026-03-27T10:31:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 12:05
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4052,6 +4052,42 @@
         </is>
       </c>
       <c r="H95" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>43.250.54.139:60000</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>1492.43</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-03-27 11:26:50</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-03-27 11:26:50</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4068,7 +4104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7688,6 +7724,42 @@
         </is>
       </c>
       <c r="H95" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>43.250.54.139:60000</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="n">
+        <v>1492.43</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-03-27 11:26:50</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-03-27 11:26:50</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9606,21 +9678,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T10:31:30.075994</t>
+          <t>2026-03-27T11:26:50.407037</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2655367231638418</v>
+        <v>0.2696629213483146</v>
       </c>
     </row>
     <row r="3">
@@ -9841,7 +9913,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -9851,7 +9923,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
@@ -9911,7 +9983,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="10">
@@ -9922,7 +9994,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T10:31:30</t>
+          <t>2026-03-27T11:26:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 13:41
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4088,6 +4088,82 @@
         </is>
       </c>
       <c r="H96" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>82.146.58.184:1080</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>🇷🇺 Россия</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1087.01</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>187.251.224.167:8081</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="n">
+        <v>2974.85</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4104,7 +4180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7760,6 +7836,82 @@
         </is>
       </c>
       <c r="H96" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>82.146.58.184:1080</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>🇷🇺 Россия</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1087.01</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>187.251.224.167:8081</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="n">
+        <v>2974.85</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -7832,7 +7984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7912,6 +8064,46 @@
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>82.146.58.184:1080</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>🇷🇺 Россия</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1087.01</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-03-27 12:05:22</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -9678,21 +9870,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D2" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T11:26:50.407037</t>
+          <t>2026-03-27T12:05:22.340555</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2696629213483146</v>
+        <v>0.2737430167597765</v>
       </c>
     </row>
     <row r="3">
@@ -9705,21 +9897,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T08:36:11.781100</t>
+          <t>2026-03-27T12:05:22.338434</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1020408163265306</v>
+        <v>0.1081081081081081</v>
       </c>
     </row>
     <row r="4">
@@ -9913,7 +10105,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3">
@@ -9923,7 +10115,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4">
@@ -9943,7 +10135,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -9983,7 +10175,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="10">
@@ -9994,7 +10186,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T11:26:50</t>
+          <t>2026-03-27T12:05:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 14:37
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4164,6 +4164,42 @@
         </is>
       </c>
       <c r="H98" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>113.11.36.205:30226</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="n">
+        <v>1097.82</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-03-27 13:41:52</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2026-03-27 13:41:52</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4180,7 +4216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H98"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7912,6 +7948,42 @@
         </is>
       </c>
       <c r="H98" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>113.11.36.205:30226</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="n">
+        <v>1097.82</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-03-27 13:41:52</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2026-03-27 13:41:52</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9870,21 +9942,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D2" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T12:05:22.340555</t>
+          <t>2026-03-27T13:41:52.923378</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2737430167597765</v>
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="3">
@@ -10105,7 +10177,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3">
@@ -10115,7 +10187,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -10175,7 +10247,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10">
@@ -10186,7 +10258,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T12:05:22</t>
+          <t>2026-03-27T13:41:52</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 15:32
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4200,6 +4200,202 @@
         </is>
       </c>
       <c r="H99" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>185.114.73.2:1080</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>🇪🇺 Европа</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1596.77</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>45.136.130.191:8453</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>313.37</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>45.140.147.155:1082</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>531.15</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>38.34.179.6:8449</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>720.92</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>167.71.196.28:8080</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="n">
+        <v>1125.33</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4216,7 +4412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7984,6 +8180,202 @@
         </is>
       </c>
       <c r="H99" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>185.114.73.2:1080</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>🇪🇺 Европа</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1596.77</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>45.136.130.191:8453</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>313.37</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>45.140.147.155:1082</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>531.15</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>38.34.179.6:8449</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>720.92</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>167.71.196.28:8080</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="n">
+        <v>1125.33</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -8192,7 +8584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9384,6 +9776,82 @@
         </is>
       </c>
       <c r="H30" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>38.34.179.6:8449</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>720.92</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>167.71.196.28:8080</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>1125.33</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9400,7 +9868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9876,6 +10344,46 @@
         </is>
       </c>
       <c r="H12" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>45.136.130.191:8453</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>313.37</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-03-27 14:38:03</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -9942,21 +10450,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T13:41:52.923378</t>
+          <t>2026-03-27T14:38:03.397046</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2777777777777778</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="3">
@@ -9969,21 +10477,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T12:05:22.338434</t>
+          <t>2026-03-27T14:38:03.393809</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1258278145695364</v>
       </c>
     </row>
     <row r="4">
@@ -10177,7 +10685,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3">
@@ -10187,7 +10695,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4">
@@ -10197,7 +10705,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -10207,7 +10715,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -10217,7 +10725,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -10247,7 +10755,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10">
@@ -10258,7 +10766,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T13:41:52</t>
+          <t>2026-03-27T14:38:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 16:31
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4396,6 +4396,42 @@
         </is>
       </c>
       <c r="H104" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>45.175.59.2:61950</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="n">
+        <v>2286.16</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>2026-03-27 15:32:32</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026-03-27 15:32:32</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4412,7 +4448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8376,6 +8412,42 @@
         </is>
       </c>
       <c r="H104" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>45.175.59.2:61950</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="n">
+        <v>2286.16</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>2026-03-27 15:32:32</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>2026-03-27 15:32:32</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -10450,21 +10522,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T14:38:03.397046</t>
+          <t>2026-03-27T15:32:32.341806</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2896174863387978</v>
       </c>
     </row>
     <row r="3">
@@ -10685,7 +10757,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3">
@@ -10695,7 +10767,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4">
@@ -10755,7 +10827,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="10">
@@ -10766,7 +10838,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T14:38:03</t>
+          <t>2026-03-27T15:32:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 17:31
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4432,6 +4432,86 @@
         </is>
       </c>
       <c r="H105" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>38.145.218.104:8449</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>2074.82</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>222.184.48.242:22222</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>2167.52</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4448,7 +4528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8448,6 +8528,86 @@
         </is>
       </c>
       <c r="H105" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>38.145.218.104:8449</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>2074.82</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>222.184.48.242:22222</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>2167.52</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -8656,7 +8816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9926,6 +10086,46 @@
       <c r="H32" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>38.145.218.104:8449</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2074.82</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-03-27 16:32:08</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -10522,21 +10722,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D2" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T15:32:32.341806</t>
+          <t>2026-03-27T16:32:08.921490</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2896174863387978</v>
+        <v>0.2934782608695652</v>
       </c>
     </row>
     <row r="3">
@@ -10549,21 +10749,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T14:38:03.393809</t>
+          <t>2026-03-27T16:32:08.919776</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1258278145695364</v>
+        <v>0.131578947368421</v>
       </c>
     </row>
     <row r="4">
@@ -10757,7 +10957,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3">
@@ -10767,7 +10967,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4">
@@ -10827,7 +11027,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="10">
@@ -10838,7 +11038,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T15:32:32</t>
+          <t>2026-03-27T16:32:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 18:31
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4514,6 +4514,86 @@
       <c r="H107" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>38.145.208.189:8449</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>207.75</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>38.145.220.188:8452</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>1612.94</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:H109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8610,6 +8690,86 @@
       <c r="H107" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>38.145.208.189:8449</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>207.75</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>38.145.220.188:8452</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>1612.94</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -8816,7 +8976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10124,6 +10284,46 @@
         </is>
       </c>
       <c r="H33" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>38.145.220.188:8452</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1612.94</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -10140,7 +10340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10656,6 +10856,46 @@
         </is>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>38.145.208.189:8449</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>207.75</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-03-27 17:31:32</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -10749,21 +10989,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T16:32:08.919776</t>
+          <t>2026-03-27T17:31:32.342241</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G3" t="n">
-        <v>0.131578947368421</v>
+        <v>0.1428571428571428</v>
       </c>
     </row>
     <row r="4">
@@ -10957,7 +11197,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3">
@@ -10967,7 +11207,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4">
@@ -10977,7 +11217,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -10987,7 +11227,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -10997,7 +11237,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -11027,7 +11267,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10">
@@ -11038,7 +11278,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T16:32:08</t>
+          <t>2026-03-27T17:31:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 19:26
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4594,6 +4594,118 @@
       <c r="H109" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8127</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="n">
+        <v>2751.32</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>38.34.179.173:8452</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1713.91</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>195.158.8.123:3128</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="n">
+        <v>2631.75</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8770,6 +8882,118 @@
       <c r="H109" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>158.160.215.167:8127</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="n">
+        <v>2751.32</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>38.34.179.173:8452</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1713.91</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>195.158.8.123:3128</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="n">
+        <v>2631.75</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -8976,7 +9200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10324,6 +10548,46 @@
         </is>
       </c>
       <c r="H34" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>38.34.179.173:8452</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1713.91</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-03-27 18:32:06</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -10962,21 +11226,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D2" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T16:32:08.921490</t>
+          <t>2026-03-27T18:32:06.856309</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2934782608695652</v>
+        <v>0.2972972972972973</v>
       </c>
     </row>
     <row r="3">
@@ -10989,21 +11253,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T17:31:32.342241</t>
+          <t>2026-03-27T18:32:06.854682</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1538461538461539</v>
       </c>
     </row>
     <row r="4">
@@ -11197,7 +11461,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3">
@@ -11207,7 +11471,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
@@ -11227,7 +11491,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -11267,7 +11531,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="10">
@@ -11278,7 +11542,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T17:31:32</t>
+          <t>2026-03-27T18:32:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 19:59
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4704,6 +4704,42 @@
         </is>
       </c>
       <c r="H112" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>165.16.27.42:1981</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="n">
+        <v>2549.81</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:26:37</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:26:37</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4720,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H112"/>
+  <dimension ref="A1:H113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8992,6 +9028,42 @@
         </is>
       </c>
       <c r="H112" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>165.16.27.42:1981</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="n">
+        <v>2549.81</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:26:37</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:26:37</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -11226,21 +11298,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D2" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T18:32:06.856309</t>
+          <t>2026-03-27T19:26:37.354160</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2972972972972973</v>
+        <v>0.3010752688172043</v>
       </c>
     </row>
     <row r="3">
@@ -11461,7 +11533,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -11471,7 +11543,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4">
@@ -11531,7 +11603,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10">
@@ -11542,7 +11614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T18:32:06</t>
+          <t>2026-03-27T19:26:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 20:52
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H113"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4740,6 +4740,114 @@
         </is>
       </c>
       <c r="H113" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>49.156.44.115:8080</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="n">
+        <v>2849.97</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>203.146.80.102:8080</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="n">
+        <v>1701.01</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>181.78.49.177:999</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="n">
+        <v>2577.3</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4756,7 +4864,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H113"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9064,6 +9172,114 @@
         </is>
       </c>
       <c r="H113" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>49.156.44.115:8080</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="n">
+        <v>2849.97</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>203.146.80.102:8080</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="n">
+        <v>1701.01</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>181.78.49.177:999</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="n">
+        <v>2577.3</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-03-27 19:59:56</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -11298,21 +11514,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D2" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T19:26:37.354160</t>
+          <t>2026-03-27T19:59:56.956951</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3010752688172043</v>
+        <v>0.3085106382978723</v>
       </c>
     </row>
     <row r="3">
@@ -11325,21 +11541,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T18:32:06.854682</t>
+          <t>2026-03-27T19:59:56.953130</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1592356687898089</v>
       </c>
     </row>
     <row r="4">
@@ -11533,7 +11749,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3">
@@ -11543,7 +11759,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
@@ -11603,7 +11819,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10">
@@ -11614,7 +11830,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T19:26:37</t>
+          <t>2026-03-27T19:59:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 21:28
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4848,6 +4848,154 @@
         </is>
       </c>
       <c r="H116" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>185.76.240.165:10001</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="n">
+        <v>1217.74</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>38.145.208.220:8451</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1092.47</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>185.76.241.111:10001</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="n">
+        <v>1059.19</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>147.75.34.105:443</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="n">
+        <v>2085.95</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -4864,7 +5012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9280,6 +9428,154 @@
         </is>
       </c>
       <c r="H116" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>185.76.240.165:10001</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="n">
+        <v>1217.74</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>38.145.208.220:8451</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1092.47</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>185.76.241.111:10001</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="n">
+        <v>1059.19</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>147.75.34.105:443</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="n">
+        <v>2085.95</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -9488,7 +9784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10876,6 +11172,118 @@
         </is>
       </c>
       <c r="H35" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>185.76.240.165:10001</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>1217.74</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>38.145.208.220:8451</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1092.47</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>185.76.241.111:10001</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>1059.19</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-03-27 20:52:29</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -11514,21 +11922,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T19:59:56.956951</t>
+          <t>2026-03-27T20:52:29.059938</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3085106382978723</v>
+        <v>0.3121693121693122</v>
       </c>
     </row>
     <row r="3">
@@ -11541,21 +11949,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T19:59:56.953130</t>
+          <t>2026-03-27T20:52:29.058072</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1592356687898089</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="4">
@@ -11749,7 +12157,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3">
@@ -11759,7 +12167,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4">
@@ -11779,7 +12187,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -11819,7 +12227,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>329</v>
+        <v>333</v>
       </c>
     </row>
     <row r="10">
@@ -11830,7 +12238,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T19:59:56</t>
+          <t>2026-03-27T20:52:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 22:00
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4996,6 +4996,42 @@
         </is>
       </c>
       <c r="H120" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>65.21.201.149:8080</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="n">
+        <v>1732.18</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>2026-03-27 21:29:12</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-03-27 21:29:12</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5012,7 +5048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9576,6 +9612,42 @@
         </is>
       </c>
       <c r="H120" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>65.21.201.149:8080</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="n">
+        <v>1732.18</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>2026-03-27 21:29:12</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-03-27 21:29:12</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -11922,21 +11994,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D2" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T20:52:29.059938</t>
+          <t>2026-03-27T21:29:12.133032</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3121693121693122</v>
+        <v>0.3157894736842105</v>
       </c>
     </row>
     <row r="3">
@@ -12157,7 +12229,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -12167,7 +12239,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4">
@@ -12227,7 +12299,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10">
@@ -12238,7 +12310,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T20:52:29</t>
+          <t>2026-03-27T21:29:12</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 22:47
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5032,6 +5032,222 @@
         </is>
       </c>
       <c r="H121" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>200.69.83.203:999</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="n">
+        <v>1168.51</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>185.225.40.236:8080</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="n">
+        <v>1032.74</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>185.76.240.150:10001</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="n">
+        <v>1615.68</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>223.205.57.57:8080</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="n">
+        <v>1728.81</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>122.185.198.242:7999</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="n">
+        <v>2636.64</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>103.102.14.51:1111</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="n">
+        <v>2687.42</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5048,7 +5264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9648,6 +9864,222 @@
         </is>
       </c>
       <c r="H121" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>200.69.83.203:999</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="n">
+        <v>1168.51</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>185.225.40.236:8080</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="n">
+        <v>1032.74</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>185.76.240.150:10001</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="n">
+        <v>1615.68</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>223.205.57.57:8080</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="n">
+        <v>1728.81</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>122.185.198.242:7999</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="n">
+        <v>2636.64</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>103.102.14.51:1111</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="n">
+        <v>2687.42</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:00:25</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -11994,21 +12426,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T21:29:12.133032</t>
+          <t>2026-03-27T22:00:25.302661</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3157894736842105</v>
+        <v>0.3264248704663212</v>
       </c>
     </row>
     <row r="3">
@@ -12021,21 +12453,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T20:52:29.058072</t>
+          <t>2026-03-27T22:00:25.297202</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="G3" t="n">
-        <v>0.175</v>
+        <v>0.1901840490797546</v>
       </c>
     </row>
     <row r="4">
@@ -12229,7 +12661,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3">
@@ -12239,7 +12671,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4">
@@ -12299,7 +12731,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="10">
@@ -12310,7 +12742,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T21:29:12</t>
+          <t>2026-03-27T22:00:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 23:19
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5250,6 +5250,326 @@
       <c r="H127" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>38.34.179.7:8448</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>482.52</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>38.34.179.36:8448</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>2092.59</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>38.145.220.72:8446</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>391.86</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>38.145.208.164:8446</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>386.99</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>38.145.208.186:8446</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>393.32</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>45.136.130.167:8449</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>1509.38</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>83.219.250.8:62920</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>458.11</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>38.145.218.104:8452</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>331.31</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H127"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10082,6 +10402,326 @@
       <c r="H127" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>38.34.179.7:8448</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>482.52</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>38.34.179.36:8448</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>2092.59</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>38.145.220.72:8446</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>391.86</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>38.145.208.164:8446</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>386.99</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>38.145.208.186:8446</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>393.32</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>45.136.130.167:8449</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>1509.38</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>83.219.250.8:62920</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>458.11</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>38.145.218.104:8452</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>331.31</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -10288,7 +10928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11788,6 +12428,246 @@
         </is>
       </c>
       <c r="H38" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>38.34.179.7:8448</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>482.52</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>38.34.179.36:8448</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>2092.59</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>38.145.220.72:8446</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>391.86</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>38.145.208.164:8446</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>386.99</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>45.136.130.167:8449</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1509.38</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>38.145.218.104:8452</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>331.31</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -11804,7 +12684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12360,6 +13240,86 @@
         </is>
       </c>
       <c r="H14" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>38.145.208.186:8446</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>393.32</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>83.219.250.8:62920</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>458.11</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-03-27 22:48:03</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -12453,21 +13413,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="D3" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T22:00:25.297202</t>
+          <t>2026-03-27T22:48:03.668391</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1901840490797546</v>
+        <v>0.2280701754385965</v>
       </c>
     </row>
     <row r="4">
@@ -12661,7 +13621,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3">
@@ -12671,7 +13631,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -12681,7 +13641,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -12691,7 +13651,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -12701,7 +13661,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -12731,7 +13691,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>340</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10">
@@ -12742,7 +13702,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T22:00:25</t>
+          <t>2026-03-27T22:48:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 23:50
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H135"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5570,6 +5570,42 @@
       <c r="H135" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>163.5.128.20:14270</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="n">
+        <v>1262.73</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:20:02</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:20:02</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -5584,7 +5620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H135"/>
+  <dimension ref="A1:H136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10722,6 +10758,42 @@
       <c r="H135" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>163.5.128.20:14270</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="n">
+        <v>1262.73</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:20:02</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:20:02</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -13386,21 +13458,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D2" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T22:00:25.302661</t>
+          <t>2026-03-27T23:20:02.469221</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3264248704663212</v>
+        <v>0.3298969072164948</v>
       </c>
     </row>
     <row r="3">
@@ -13621,7 +13693,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3">
@@ -13631,7 +13703,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
@@ -13691,7 +13763,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>348</v>
+        <v>349</v>
       </c>
     </row>
     <row r="10">
@@ -13702,7 +13774,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T22:48:03</t>
+          <t>2026-03-27T23:20:02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 01:05
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5604,6 +5604,162 @@
         </is>
       </c>
       <c r="H136" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>38.145.218.210:8449</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>340.75</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>38.145.208.219:8450</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>340.02</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>38.145.208.167:8445</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>657.14</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>116.171.106.15:3443</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="n">
+        <v>1516.52</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5620,7 +5776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H136"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10792,6 +10948,162 @@
         </is>
       </c>
       <c r="H136" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>38.145.218.210:8449</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>340.75</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>38.145.208.219:8450</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>340.02</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>38.145.208.167:8445</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>657.14</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>116.171.106.15:3443</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="n">
+        <v>1516.52</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -12756,7 +13068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13392,6 +13704,126 @@
         </is>
       </c>
       <c r="H16" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>38.145.218.210:8449</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>340.75</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>38.145.208.219:8450</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>340.02</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>38.145.208.167:8445</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>657.14</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-03-27 23:50:19</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -13458,21 +13890,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T23:20:02.469221</t>
+          <t>2026-03-27T23:50:19.220271</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3298969072164948</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -13485,21 +13917,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D3" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T22:48:03.668391</t>
+          <t>2026-03-27T23:50:19.218314</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2280701754385965</v>
+        <v>0.2413793103448276</v>
       </c>
     </row>
     <row r="4">
@@ -13693,7 +14125,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3">
@@ -13703,7 +14135,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4">
@@ -13713,7 +14145,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -13723,7 +14155,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -13733,7 +14165,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -13763,7 +14195,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10">
@@ -13774,7 +14206,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T23:20:02</t>
+          <t>2026-03-27T23:50:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 05:14
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5760,6 +5760,162 @@
         </is>
       </c>
       <c r="H140" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>38.145.208.234:8453</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>689.4400000000001</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>38.145.218.76:8451</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>384.97</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>38.34.179.30:8447</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>400.76</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>50.235.247.114:8085</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="n">
+        <v>2305.95</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5776,7 +5932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H140"/>
+  <dimension ref="A1:H144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11104,6 +11260,162 @@
         </is>
       </c>
       <c r="H140" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>38.145.208.234:8453</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>689.4400000000001</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>38.145.218.76:8451</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>384.97</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>38.34.179.30:8447</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>400.76</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>50.235.247.114:8085</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="n">
+        <v>2305.95</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -11312,7 +11624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13052,6 +13364,86 @@
         </is>
       </c>
       <c r="H44" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>38.145.218.76:8451</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>384.97</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>38.34.179.30:8447</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>400.76</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -13068,7 +13460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13824,6 +14216,46 @@
         </is>
       </c>
       <c r="H19" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>38.145.208.234:8453</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>689.4400000000001</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-03-28 03:45:15</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -13890,21 +14322,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-27T23:50:19.220271</t>
+          <t>2026-03-28T03:45:15.417856</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.336734693877551</v>
       </c>
     </row>
     <row r="3">
@@ -13917,21 +14349,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D3" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-27T23:50:19.218314</t>
+          <t>2026-03-28T03:45:15.415901</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2413793103448276</v>
+        <v>0.2542372881355932</v>
       </c>
     </row>
     <row r="4">
@@ -14125,7 +14557,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3">
@@ -14135,7 +14567,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4">
@@ -14145,7 +14577,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -14155,7 +14587,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6">
@@ -14165,7 +14597,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -14195,7 +14627,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10">
@@ -14206,7 +14638,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-27T23:50:19</t>
+          <t>2026-03-28T03:45:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 06:13
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H144"/>
+  <dimension ref="A1:H148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5916,6 +5916,158 @@
         </is>
       </c>
       <c r="H144" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>101.251.204.174:8080</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="n">
+        <v>1083.46</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>45.136.131.55:8453</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>893.27</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>190.12.150.244:999</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>2426.93</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>181.129.147.163:8080</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="n">
+        <v>2589.97</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -5932,7 +6084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H144"/>
+  <dimension ref="A1:H148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11416,6 +11568,158 @@
         </is>
       </c>
       <c r="H144" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>101.251.204.174:8080</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="n">
+        <v>1083.46</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>45.136.131.55:8453</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>893.27</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>190.12.150.244:999</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>2426.93</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>181.129.147.163:8080</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="n">
+        <v>2589.97</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -11624,7 +11928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13444,6 +13748,46 @@
         </is>
       </c>
       <c r="H46" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>45.136.131.55:8453</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>893.27</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-03-28 05:14:59</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -14322,21 +14666,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D2" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T03:45:15.417856</t>
+          <t>2026-03-28T05:14:59.644042</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G2" t="n">
-        <v>0.336734693877551</v>
+        <v>0.3401015228426396</v>
       </c>
     </row>
     <row r="3">
@@ -14349,21 +14693,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D3" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T03:45:15.415901</t>
+          <t>2026-03-28T05:14:59.641885</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2542372881355932</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -14557,7 +14901,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="3">
@@ -14567,7 +14911,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>143</v>
+        <v>147</v>
       </c>
     </row>
     <row r="4">
@@ -14627,7 +14971,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10">
@@ -14638,7 +14982,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T03:45:15</t>
+          <t>2026-03-28T05:14:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 07:16
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H148"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6068,6 +6068,78 @@
         </is>
       </c>
       <c r="H148" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>180.191.23.26:8081</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="n">
+        <v>2539</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>27.147.137.234:9108</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="n">
+        <v>2505.02</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6084,7 +6156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H148"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11720,6 +11792,78 @@
         </is>
       </c>
       <c r="H148" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>180.191.23.26:8081</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="n">
+        <v>2539</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>27.147.137.234:9108</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="n">
+        <v>2505.02</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2026-03-28 06:13:39</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -14666,21 +14810,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D2" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T05:14:59.644042</t>
+          <t>2026-03-28T06:13:39.592780</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3401015228426396</v>
+        <v>0.3467336683417085</v>
       </c>
     </row>
     <row r="3">
@@ -14901,7 +15045,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="3">
@@ -14911,7 +15055,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4">
@@ -14971,7 +15115,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="10">
@@ -14982,7 +15126,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T05:14:59</t>
+          <t>2026-03-28T06:13:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 07:57
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6140,6 +6140,42 @@
         </is>
       </c>
       <c r="H150" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>104.251.81.37:14270</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="n">
+        <v>2550.91</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:16:51</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:16:51</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6156,7 +6192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11864,6 +11900,42 @@
         </is>
       </c>
       <c r="H150" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>104.251.81.37:14270</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="n">
+        <v>2550.91</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:16:51</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:16:51</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -14810,21 +14882,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T06:13:39.592780</t>
+          <t>2026-03-28T07:16:51.137157</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3467336683417085</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="3">
@@ -15045,7 +15117,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
@@ -15055,7 +15127,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4">
@@ -15115,7 +15187,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="10">
@@ -15126,7 +15198,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T06:13:39</t>
+          <t>2026-03-28T07:16:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 08:52
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6178,6 +6178,46 @@
       <c r="H151" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>64.181.240.152:3128</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>234.81</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:57:19</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:57:19</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11938,6 +11978,46 @@
       <c r="H151" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>64.181.240.152:3128</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>234.81</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:57:19</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:57:19</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -12144,7 +12224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H47"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14004,6 +14084,46 @@
         </is>
       </c>
       <c r="H47" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>64.181.240.152:3128</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>234.81</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:57:19</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-03-28 07:57:19</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -14909,21 +15029,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D3" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T05:14:59.641885</t>
+          <t>2026-03-28T07:57:19.689070</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2666666666666667</v>
+        <v>0.2707182320441989</v>
       </c>
     </row>
     <row r="4">
@@ -15117,7 +15237,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
@@ -15127,7 +15247,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="4">
@@ -15147,7 +15267,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -15187,7 +15307,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="10">
@@ -15198,7 +15318,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T07:16:51</t>
+          <t>2026-03-28T07:57:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 09:31
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6216,6 +6216,46 @@
         </is>
       </c>
       <c r="H152" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>45.144.28.81:10808</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1608.33</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>2026-03-28 08:52:54</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2026-03-28 08:52:54</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -6232,7 +6272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H152"/>
+  <dimension ref="A1:H153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12016,6 +12056,46 @@
         </is>
       </c>
       <c r="H152" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>45.144.28.81:10808</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1608.33</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>2026-03-28 08:52:54</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2026-03-28 08:52:54</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -15029,21 +15109,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T07:57:19.689070</t>
+          <t>2026-03-28T08:52:54.439285</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2707182320441989</v>
+        <v>0.2747252747252747</v>
       </c>
     </row>
     <row r="4">
@@ -15237,7 +15317,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
@@ -15247,7 +15327,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4">
@@ -15307,7 +15387,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="10">
@@ -15318,7 +15398,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T07:57:19</t>
+          <t>2026-03-28T08:52:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 10:48
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6258,6 +6258,42 @@
       <c r="H153" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>103.26.176.31:8080</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="n">
+        <v>2817.18</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>2026-03-28 10:03:24</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2026-03-28 10:03:24</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -6272,7 +6308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H153"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12098,6 +12134,42 @@
       <c r="H153" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>103.26.176.31:8080</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="n">
+        <v>2817.18</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>2026-03-28 10:03:24</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2026-03-28 10:03:24</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -15082,21 +15154,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T07:16:51.137157</t>
+          <t>2026-03-28T10:03:24.579821</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G2" t="n">
-        <v>0.35</v>
+        <v>0.3532338308457711</v>
       </c>
     </row>
     <row r="3">
@@ -15317,7 +15389,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3">
@@ -15327,7 +15399,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
@@ -15387,7 +15459,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="10">
@@ -15398,7 +15470,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T08:52:54</t>
+          <t>2026-03-28T10:03:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 11:46
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H154"/>
+  <dimension ref="A1:H157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6292,6 +6292,122 @@
         </is>
       </c>
       <c r="H154" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>45.144.232.5:11741</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1163.34</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>128.199.114.189:9090</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1574.69</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>190.54.100.74:8080</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="n">
+        <v>1698.92</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6308,7 +6424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H154"/>
+  <dimension ref="A1:H157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12168,6 +12284,122 @@
         </is>
       </c>
       <c r="H154" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>45.144.232.5:11741</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1163.34</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>128.199.114.189:9090</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1574.69</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>190.54.100.74:8080</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="n">
+        <v>1698.92</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:16:32</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -15154,21 +15386,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D2" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T10:03:24.579821</t>
+          <t>2026-03-28T11:16:32.276362</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3532338308457711</v>
+        <v>0.3564356435643564</v>
       </c>
     </row>
     <row r="3">
@@ -15181,21 +15413,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D3" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T08:52:54.439285</t>
+          <t>2026-03-28T11:16:32.273858</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2747252747252747</v>
+        <v>0.2826086956521739</v>
       </c>
     </row>
     <row r="4">
@@ -15389,7 +15621,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3">
@@ -15399,7 +15631,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4">
@@ -15459,7 +15691,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="10">
@@ -15470,7 +15702,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T10:03:24</t>
+          <t>2026-03-28T11:16:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 12:23
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6408,6 +6408,122 @@
         </is>
       </c>
       <c r="H157" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>128.199.254.13:9090</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>1356.18</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>168.63.153.150:3128</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>1043.57</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>190.60.40.243:999</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="n">
+        <v>2638.71</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6424,7 +6540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12400,6 +12516,122 @@
         </is>
       </c>
       <c r="H157" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>128.199.254.13:9090</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>1356.18</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>168.63.153.150:3128</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>1043.57</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>190.60.40.243:999</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="n">
+        <v>2638.71</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -12608,7 +12840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14510,6 +14742,46 @@
       <c r="H48" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>168.63.153.150:3128</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1043.57</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-03-28 11:46:50</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -15386,21 +15658,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D2" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T11:16:32.276362</t>
+          <t>2026-03-28T11:46:50.930648</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3564356435643564</v>
+        <v>0.3627450980392157</v>
       </c>
     </row>
     <row r="3">
@@ -15413,21 +15685,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D3" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T11:16:32.273858</t>
+          <t>2026-03-28T11:46:50.925706</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2826086956521739</v>
+        <v>0.2864864864864865</v>
       </c>
     </row>
     <row r="4">
@@ -15621,7 +15893,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3">
@@ -15631,7 +15903,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4">
@@ -15651,7 +15923,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -15691,7 +15963,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="10">
@@ -15702,7 +15974,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T11:16:32</t>
+          <t>2026-03-28T11:46:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 13:31
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6524,6 +6524,42 @@
         </is>
       </c>
       <c r="H160" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>103.124.136.251:8080</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="n">
+        <v>2921.96</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>2026-03-28 12:23:58</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2026-03-28 12:23:58</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6540,7 +6576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12632,6 +12668,42 @@
         </is>
       </c>
       <c r="H160" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>103.124.136.251:8080</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="n">
+        <v>2921.96</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>2026-03-28 12:23:58</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>2026-03-28 12:23:58</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -15658,21 +15730,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T11:46:50.930648</t>
+          <t>2026-03-28T12:23:58.221391</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3627450980392157</v>
+        <v>0.3658536585365854</v>
       </c>
     </row>
     <row r="3">
@@ -15893,7 +15965,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3">
@@ -15903,7 +15975,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4">
@@ -15963,7 +16035,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="10">
@@ -15974,7 +16046,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T11:46:50</t>
+          <t>2026-03-28T12:23:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 14:06
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H161"/>
+  <dimension ref="A1:H163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6560,6 +6560,78 @@
         </is>
       </c>
       <c r="H161" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>45.174.56.21:999</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="n">
+        <v>2833.68</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>200.10.28.254:999</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="n">
+        <v>1407.51</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6576,7 +6648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H161"/>
+  <dimension ref="A1:H163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12704,6 +12776,78 @@
         </is>
       </c>
       <c r="H161" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>45.174.56.21:999</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="n">
+        <v>2833.68</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>200.10.28.254:999</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="n">
+        <v>1407.51</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>2026-03-28 13:32:09</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -15730,21 +15874,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T12:23:58.221391</t>
+          <t>2026-03-28T13:32:09.224735</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3658536585365854</v>
+        <v>0.3719806763285024</v>
       </c>
     </row>
     <row r="3">
@@ -15965,7 +16109,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3">
@@ -15975,7 +16119,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4">
@@ -16035,7 +16179,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10">
@@ -16046,7 +16190,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T12:23:58</t>
+          <t>2026-03-28T13:32:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 14:30
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:H165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6632,6 +6632,78 @@
         </is>
       </c>
       <c r="H163" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>221.202.27.194:10809</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="n">
+        <v>1009.62</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2.56.173.45:10808</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="n">
+        <v>1736.17</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -6648,7 +6720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H163"/>
+  <dimension ref="A1:H165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12848,6 +12920,78 @@
         </is>
       </c>
       <c r="H163" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>221.202.27.194:10809</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="n">
+        <v>1009.62</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2.56.173.45:10808</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="n">
+        <v>1736.17</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:06:59</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -15874,21 +16018,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D2" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T13:32:09.224735</t>
+          <t>2026-03-28T14:06:59.478933</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3719806763285024</v>
+        <v>0.3779904306220095</v>
       </c>
     </row>
     <row r="3">
@@ -16109,7 +16253,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -16119,7 +16263,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4">
@@ -16179,7 +16323,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>376</v>
+        <v>378</v>
       </c>
     </row>
     <row r="10">
@@ -16190,7 +16334,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T13:32:09</t>
+          <t>2026-03-28T14:06:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 14:34
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H165"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6706,6 +6706,46 @@
       <c r="H165" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>180.250.219.58:53281</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>1318.51</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:31:30</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:31:30</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H165"/>
+  <dimension ref="A1:H166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12994,6 +13034,46 @@
       <c r="H165" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>180.250.219.58:53281</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>1318.51</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:31:30</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:31:30</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -16045,21 +16125,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T11:46:50.925706</t>
+          <t>2026-03-28T14:31:30.012447</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2864864864864865</v>
+        <v>0.2903225806451613</v>
       </c>
     </row>
     <row r="4">
@@ -16253,7 +16333,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3">
@@ -16263,7 +16343,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4">
@@ -16323,7 +16403,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10">
@@ -16334,7 +16414,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T14:06:59</t>
+          <t>2026-03-28T14:31:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 14:50
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6746,6 +6746,158 @@
       <c r="H166" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>177.234.217.88:999</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>482.1</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>84.32.6.251:49146</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="n">
+        <v>2907.42</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>103.30.31.202:20326</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="n">
+        <v>2162.41</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>64.227.76.27:1080</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>833.2</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H166"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13074,6 +13226,158 @@
       <c r="H166" t="inlineStr">
         <is>
           <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>177.234.217.88:999</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>482.1</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>84.32.6.251:49146</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="n">
+        <v>2907.42</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>103.30.31.202:20326</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="n">
+        <v>2162.41</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>64.227.76.27:1080</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>833.2</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
         </is>
       </c>
     </row>
@@ -13280,7 +13584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15220,6 +15524,86 @@
         </is>
       </c>
       <c r="H49" t="inlineStr">
+        <is>
+          <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>177.234.217.88:999</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>482.1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>64.227.76.27:1080</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>833.2</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:35:01</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
         </is>
@@ -16098,21 +16482,21 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D2" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-28T14:06:59.478933</t>
+          <t>2026-03-28T14:35:01.519411</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3779904306220095</v>
+        <v>0.3867924528301887</v>
       </c>
     </row>
     <row r="3">
@@ -16125,21 +16509,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D3" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T14:31:30.012447</t>
+          <t>2026-03-28T14:35:01.512197</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2903225806451613</v>
+        <v>0.2941176470588235</v>
       </c>
     </row>
     <row r="4">
@@ -16333,7 +16717,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3">
@@ -16343,7 +16727,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4">
@@ -16363,7 +16747,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
@@ -16403,7 +16787,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="10">
@@ -16414,7 +16798,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T14:31:30</t>
+          <t>2026-03-28T14:35:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 14:58
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:H174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6898,6 +6898,162 @@
       <c r="H170" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>194.59.204.87:9080</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>808.4400000000001</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>38.145.208.185:8444</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="n">
+        <v>1944.33</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>38.34.179.69:8453</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>955.63</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>38.145.208.229:8450</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>535.62</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -6912,7 +7068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H170"/>
+  <dimension ref="A1:H174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13378,6 +13534,162 @@
       <c r="H170" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>194.59.204.87:9080</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>808.4400000000001</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>38.145.208.185:8444</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>❓ Неизвестно</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="n">
+        <v>1944.33</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>38.34.179.69:8453</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>955.63</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>38.145.208.229:8450</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>535.62</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -13584,7 +13896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15606,6 +15918,86 @@
       <c r="H51" t="inlineStr">
         <is>
           <t>thespeedx_http</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>194.59.204.87:9080</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>808.4400000000001</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>38.34.179.69:8453</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>🇺🇸 США</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>955.63</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>proxymania</t>
         </is>
       </c>
     </row>
@@ -15620,7 +16012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16416,6 +16808,46 @@
         </is>
       </c>
       <c r="H20" t="inlineStr">
+        <is>
+          <t>proxymania</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>38.145.208.229:8450</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>✅ Да</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>🌍 Глобальный</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>535.62</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-03-28 14:50:45</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>proxymania</t>
         </is>
@@ -16509,21 +16941,21 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D3" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-28T14:35:01.512197</t>
+          <t>2026-03-28T14:50:45.434937</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G3" t="n">
-        <v>0.2941176470588235</v>
+        <v>0.3089005235602094</v>
       </c>
     </row>
     <row r="4">
@@ -16717,7 +17149,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3">
@@ -16727,7 +17159,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4">
@@ -16737,7 +17169,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -16747,7 +17179,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -16757,7 +17189,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -16787,7 +17219,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>383</v>
+        <v>387</v>
       </c>
     </row>
     <row r="10">
@@ -16798,7 +17230,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T14:35:01</t>
+          <t>2026-03-28T14:50:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Report update: 15:08
</commit_message>
<xml_diff>
--- a/reports/proxy_report.xlsx
+++ b/reports/proxy_report.xlsx
@@ -1507,7 +1507,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1318.51</v>
+        <v>1220.62</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-03-28 14:31:30</t>
+          <t>2026-03-28 15:04:44</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1318.51</v>
+        <v>1220.62</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -2928,7 +2928,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-03-28 14:31:30</t>
+          <t>2026-03-28 15:04:44</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-03-28T14:58:49</t>
+          <t>2026-03-28T15:04:44</t>
         </is>
       </c>
     </row>

</xml_diff>